<commit_message>
working visualization of X and cap inc
</commit_message>
<xml_diff>
--- a/DATA/Vaccine_price_data.xlsx
+++ b/DATA/Vaccine_price_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/5e6b18ad1acc1266/Desktop/Vaccine_Tender/DATA/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="162" documentId="13_ncr:1_{5713AA50-68F1-4433-87EB-33DE309D44C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3A15BE83-0466-4F3D-AD6E-62F521E580CC}"/>
+  <xr:revisionPtr revIDLastSave="164" documentId="13_ncr:1_{5713AA50-68F1-4433-87EB-33DE309D44C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C18B6798-22FC-4C6E-BE00-811C6018706E}"/>
   <bookViews>
-    <workbookView xWindow="13550" yWindow="-110" windowWidth="38620" windowHeight="21100" firstSheet="1" activeTab="9" xr2:uid="{4E5F4A35-5A78-441E-8AE9-B1CCE3EF1506}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{4E5F4A35-5A78-441E-8AE9-B1CCE3EF1506}"/>
   </bookViews>
   <sheets>
     <sheet name="vaccine-producer list" sheetId="70" r:id="rId1"/>
@@ -1344,9 +1344,7 @@
         <v>1</v>
       </c>
       <c r="E4" s="27"/>
-      <c r="F4" s="27">
-        <v>1</v>
-      </c>
+      <c r="F4" s="27"/>
       <c r="G4" s="27"/>
       <c r="H4" s="27"/>
       <c r="I4" s="27"/>
@@ -1359,7 +1357,7 @@
       <c r="P4" s="29"/>
       <c r="Q4">
         <f t="shared" si="0"/>
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
@@ -1800,7 +1798,7 @@
       </c>
       <c r="F19" s="2">
         <f t="shared" si="1"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G19" s="2">
         <f t="shared" si="1"/>

</xml_diff>